<commit_message>
Update treatment plan report to include monthly value with discounts
Add a new column to the treatment plan export that calculates the net monthly value after applying discounts.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: f9fbcc8a-3df4-48a5-aab2-6ba2c3cbfeed
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: 592978e9-d90e-4324-825a-5c598b0cf096
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/c324e96a-0238-47f5-a609-b6a2412bcc0e/f9fbcc8a-3df4-48a5-aab2-6ba2c3cbfeed/frYyIrq
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/exports/planos-de-tratamento.xlsx
+++ b/exports/planos-de-tratamento.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="397" uniqueCount="151">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="428" uniqueCount="158">
   <si>
     <t>ID</t>
   </si>
@@ -60,6 +60,9 @@
     <t>Técnicas</t>
   </si>
   <si>
+    <t>Valor mensal líq. (R$)</t>
+  </si>
+  <si>
     <t>Valor total (R$)</t>
   </si>
   <si>
@@ -93,6 +96,9 @@
     <t>1x/semana</t>
   </si>
   <si>
+    <t>170.00</t>
+  </si>
+  <si>
     <t>Clarisse Helms Couto</t>
   </si>
   <si>
@@ -123,6 +129,9 @@
     <t>Marta Wille Schuch</t>
   </si>
   <si>
+    <t>0</t>
+  </si>
+  <si>
     <t>Luciana Grellert</t>
   </si>
   <si>
@@ -138,6 +147,9 @@
     <t>94817898020</t>
   </si>
   <si>
+    <t>160.00</t>
+  </si>
+  <si>
     <t>Maria Isabel Roveré</t>
   </si>
   <si>
@@ -166,6 +178,9 @@
   </si>
   <si>
     <t>(53) 99112-7696</t>
+  </si>
+  <si>
+    <t>210.00</t>
   </si>
   <si>
     <t>Roberta Bartz Kneib</t>
@@ -194,10 +209,16 @@
     <t>Exercícios ativos de alongamento e fortalecimento de MMII, MMSS, abdomen e tronco</t>
   </si>
   <si>
+    <t>200.00</t>
+  </si>
+  <si>
     <t>Vilda Soares dos Santos</t>
   </si>
   <si>
     <t>30210364068</t>
+  </si>
+  <si>
+    <t>220.00</t>
   </si>
   <si>
     <t>Vera Souza</t>
@@ -881,7 +902,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:T30"/>
+  <dimension ref="A1:U30"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="6" customWidth="1"/>
@@ -897,13 +918,14 @@
     <col min="13" max="13" width="22" customWidth="1"/>
     <col min="14" max="14" width="40" customWidth="1"/>
     <col min="15" max="15" width="30" customWidth="1"/>
-    <col min="16" max="16" width="16" style="2" customWidth="1"/>
-    <col min="17" max="18" width="18" style="3" customWidth="1"/>
-    <col min="19" max="19" width="8" customWidth="1"/>
-    <col min="20" max="20" width="18" style="3" customWidth="1"/>
+    <col min="16" max="16" width="18" style="2" customWidth="1"/>
+    <col min="17" max="17" width="16" style="2" customWidth="1"/>
+    <col min="18" max="19" width="18" style="3" customWidth="1"/>
+    <col min="20" max="20" width="8" customWidth="1"/>
+    <col min="21" max="21" width="18" style="3" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="22" customHeight="1" spans="1:20" s="4" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" ht="22" customHeight="1" spans="1:21" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
@@ -952,40 +974,43 @@
       <c r="P1" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="7" t="s">
+      <c r="Q1" s="6" t="s">
         <v>16</v>
       </c>
       <c r="R1" s="7" t="s">
         <v>17</v>
       </c>
-      <c r="S1" s="4" t="s">
+      <c r="S1" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="T1" s="7" t="s">
+      <c r="T1" s="4" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="2" spans="1:20" x14ac:dyDescent="0.25">
+      <c r="U1" s="7" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="2" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>76</v>
       </c>
       <c r="B2" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C2" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="D2" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="E2" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="F2" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="G2" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="I2">
         <v>12</v>
@@ -994,38 +1019,41 @@
         <v>46113</v>
       </c>
       <c r="K2" s="1"/>
-      <c r="P2" s="2">
-        <v>370</v>
-      </c>
-      <c r="Q2" s="3">
+      <c r="P2" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q2" s="2">
+        <v>2240</v>
+      </c>
+      <c r="R2" s="3">
         <v>46141.084351006946</v>
       </c>
-      <c r="R2" s="3"/>
-      <c r="S2">
+      <c r="S2" s="3"/>
+      <c r="T2">
         <v>3</v>
       </c>
-      <c r="T2" s="3">
+      <c r="U2" s="3">
         <v>46141.08342016204</v>
       </c>
     </row>
-    <row r="3" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>75</v>
       </c>
       <c r="B3" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="C3" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="D3" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="F3" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="G3" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="I3">
         <v>12</v>
@@ -1034,41 +1062,44 @@
         <v>46140</v>
       </c>
       <c r="K3" s="1"/>
-      <c r="P3" s="2">
-        <v>290</v>
-      </c>
-      <c r="Q3" s="3">
+      <c r="P3" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q3" s="2">
+        <v>2160</v>
+      </c>
+      <c r="R3" s="3">
         <v>46141.10788350695</v>
       </c>
-      <c r="R3" s="3"/>
-      <c r="S3">
+      <c r="S3" s="3"/>
+      <c r="T3">
         <v>3</v>
       </c>
-      <c r="T3" s="3">
+      <c r="U3" s="3">
         <v>46140.96744306713</v>
       </c>
     </row>
-    <row r="4" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>74</v>
       </c>
       <c r="B4" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C4" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="D4" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="E4" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="F4" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="G4" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="I4">
         <v>12</v>
@@ -1078,113 +1109,122 @@
       </c>
       <c r="K4" s="1"/>
       <c r="L4" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="N4" t="s">
-        <v>31</v>
-      </c>
-      <c r="P4" s="2">
-        <v>290</v>
-      </c>
-      <c r="Q4" s="3">
+        <v>33</v>
+      </c>
+      <c r="P4" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q4" s="2">
+        <v>2160</v>
+      </c>
+      <c r="R4" s="3">
         <v>46141.03350622686</v>
       </c>
-      <c r="R4" s="3"/>
-      <c r="S4">
+      <c r="S4" s="3"/>
+      <c r="T4">
         <v>3</v>
       </c>
-      <c r="T4" s="3">
+      <c r="U4" s="3">
         <v>46140.044840891205</v>
       </c>
     </row>
-    <row r="5" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>73</v>
       </c>
       <c r="B5" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="C5" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="D5" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="F5" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="G5" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="J5" s="1">
         <v>46139</v>
       </c>
       <c r="K5" s="1"/>
       <c r="M5" t="s">
-        <v>35</v>
-      </c>
-      <c r="P5" s="2">
+        <v>37</v>
+      </c>
+      <c r="P5" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="Q5" s="2">
         <v>80</v>
       </c>
-      <c r="Q5" s="3"/>
       <c r="R5" s="3"/>
-      <c r="S5">
+      <c r="S5" s="3"/>
+      <c r="T5">
         <v>3</v>
       </c>
-      <c r="T5" s="3">
+      <c r="U5" s="3">
         <v>46140.04426408565</v>
       </c>
     </row>
-    <row r="6" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>72</v>
       </c>
       <c r="B6" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="C6" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="D6" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="F6" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="J6" s="1">
         <v>46137</v>
       </c>
       <c r="K6" s="1"/>
-      <c r="P6" s="2">
+      <c r="P6" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="Q6" s="2">
         <v>80</v>
       </c>
-      <c r="Q6" s="3"/>
       <c r="R6" s="3"/>
-      <c r="S6">
+      <c r="S6" s="3"/>
+      <c r="T6">
         <v>3</v>
       </c>
-      <c r="T6" s="3">
+      <c r="U6" s="3">
         <v>46137.85026872685</v>
       </c>
     </row>
-    <row r="7" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>71</v>
       </c>
       <c r="B7" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="C7" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="D7" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="F7" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="G7" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="I7">
         <v>12</v>
@@ -1196,51 +1236,54 @@
         <v>46478</v>
       </c>
       <c r="M7" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="N7" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="O7" t="s">
-        <v>23</v>
-      </c>
-      <c r="P7" s="2">
-        <v>160</v>
-      </c>
-      <c r="Q7" s="3">
-        <v>46140.47296136574</v>
+        <v>24</v>
+      </c>
+      <c r="P7" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="Q7" s="2">
+        <v>2030</v>
       </c>
       <c r="R7" s="3">
         <v>46140.47296136574</v>
       </c>
-      <c r="S7">
+      <c r="S7" s="3">
+        <v>46140.47296136574</v>
+      </c>
+      <c r="T7">
         <v>3</v>
       </c>
-      <c r="T7" s="3">
+      <c r="U7" s="3">
         <v>46133.76320414351</v>
       </c>
     </row>
-    <row r="8" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>70</v>
       </c>
       <c r="B8" t="s">
-        <v>41</v>
+        <v>45</v>
       </c>
       <c r="C8" t="s">
-        <v>42</v>
+        <v>46</v>
       </c>
       <c r="D8" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="E8" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="F8" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="G8" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="H8">
         <v>10</v>
@@ -1250,85 +1293,91 @@
       </c>
       <c r="K8" s="1"/>
       <c r="M8" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="N8" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="O8" t="s">
-        <v>45</v>
-      </c>
-      <c r="P8" s="2">
+        <v>49</v>
+      </c>
+      <c r="P8" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="Q8" s="2">
         <v>700</v>
       </c>
-      <c r="Q8" s="3"/>
       <c r="R8" s="3"/>
-      <c r="S8">
+      <c r="S8" s="3"/>
+      <c r="T8">
         <v>3</v>
       </c>
-      <c r="T8" s="3">
+      <c r="U8" s="3">
         <v>46133.76146310185</v>
       </c>
     </row>
-    <row r="9" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>68</v>
       </c>
       <c r="B9" t="s">
-        <v>46</v>
+        <v>50</v>
       </c>
       <c r="C9" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="D9" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="F9" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="G9" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="J9" s="1">
         <v>46131</v>
       </c>
       <c r="K9" s="1"/>
       <c r="N9" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="O9" t="s">
-        <v>23</v>
-      </c>
-      <c r="P9" s="2">
+        <v>24</v>
+      </c>
+      <c r="P9" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="Q9" s="2">
         <v>40</v>
       </c>
-      <c r="Q9" s="3"/>
       <c r="R9" s="3"/>
-      <c r="S9">
+      <c r="S9" s="3"/>
+      <c r="T9">
         <v>3</v>
       </c>
-      <c r="T9" s="3">
+      <c r="U9" s="3">
         <v>46131.60485847222</v>
       </c>
     </row>
-    <row r="10" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>67</v>
       </c>
       <c r="B10" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="C10" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="D10" t="s">
-        <v>50</v>
+        <v>54</v>
       </c>
       <c r="F10" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="G10" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="I10">
         <v>12</v>
@@ -1340,48 +1389,51 @@
         <v>46478</v>
       </c>
       <c r="M10" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="N10" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="O10" t="s">
-        <v>23</v>
-      </c>
-      <c r="P10" s="2">
-        <v>210</v>
-      </c>
-      <c r="Q10" s="3">
-        <v>46140.48729346065</v>
+        <v>24</v>
+      </c>
+      <c r="P10" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="Q10" s="2">
+        <v>2630</v>
       </c>
       <c r="R10" s="3">
         <v>46140.48729346065</v>
       </c>
-      <c r="S10">
+      <c r="S10" s="3">
+        <v>46140.48729346065</v>
+      </c>
+      <c r="T10">
         <v>3</v>
       </c>
-      <c r="T10" s="3">
+      <c r="U10" s="3">
         <v>46131.60328072916</v>
       </c>
     </row>
-    <row r="11" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>66</v>
       </c>
       <c r="B11" t="s">
-        <v>51</v>
+        <v>56</v>
       </c>
       <c r="C11" t="s">
-        <v>52</v>
+        <v>57</v>
       </c>
       <c r="D11" t="s">
-        <v>53</v>
+        <v>58</v>
       </c>
       <c r="F11" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="G11" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="I11">
         <v>12</v>
@@ -1393,48 +1445,51 @@
         <v>46478</v>
       </c>
       <c r="M11" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="N11" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="O11" t="s">
-        <v>23</v>
-      </c>
-      <c r="P11" s="2">
-        <v>160</v>
-      </c>
-      <c r="Q11" s="3">
-        <v>46140.48692473379</v>
+        <v>24</v>
+      </c>
+      <c r="P11" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="Q11" s="2">
+        <v>2030</v>
       </c>
       <c r="R11" s="3">
         <v>46140.48692473379</v>
       </c>
-      <c r="S11">
+      <c r="S11" s="3">
+        <v>46140.48692473379</v>
+      </c>
+      <c r="T11">
         <v>3</v>
       </c>
-      <c r="T11" s="3">
+      <c r="U11" s="3">
         <v>46131.596154074075</v>
       </c>
     </row>
-    <row r="12" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>65</v>
       </c>
       <c r="B12" t="s">
-        <v>54</v>
+        <v>59</v>
       </c>
       <c r="C12" t="s">
-        <v>55</v>
+        <v>60</v>
       </c>
       <c r="D12" t="s">
-        <v>56</v>
+        <v>61</v>
       </c>
       <c r="F12" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="G12" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="I12">
         <v>12</v>
@@ -1446,48 +1501,51 @@
         <v>46478</v>
       </c>
       <c r="M12" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="N12" t="s">
-        <v>57</v>
+        <v>62</v>
       </c>
       <c r="O12" t="s">
-        <v>58</v>
-      </c>
-      <c r="P12" s="2">
-        <v>200</v>
-      </c>
-      <c r="Q12" s="3">
-        <v>46140.4865587963</v>
+        <v>63</v>
+      </c>
+      <c r="P12" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="Q12" s="2">
+        <v>2620</v>
       </c>
       <c r="R12" s="3">
         <v>46140.4865587963</v>
       </c>
-      <c r="S12">
+      <c r="S12" s="3">
+        <v>46140.4865587963</v>
+      </c>
+      <c r="T12">
         <v>3</v>
       </c>
-      <c r="T12" s="3">
+      <c r="U12" s="3">
         <v>46131.59445065972</v>
       </c>
     </row>
-    <row r="13" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>64</v>
       </c>
       <c r="B13" t="s">
-        <v>59</v>
+        <v>65</v>
       </c>
       <c r="C13" t="s">
-        <v>60</v>
+        <v>66</v>
       </c>
       <c r="D13" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="F13" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="G13" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="I13">
         <v>12</v>
@@ -1499,45 +1557,48 @@
         <v>46505</v>
       </c>
       <c r="N13" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="O13" t="s">
-        <v>23</v>
-      </c>
-      <c r="P13" s="2">
-        <v>220</v>
-      </c>
-      <c r="Q13" s="3">
-        <v>46140.48586303241</v>
+        <v>24</v>
+      </c>
+      <c r="P13" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="Q13" s="2">
+        <v>2640</v>
       </c>
       <c r="R13" s="3">
         <v>46140.48586303241</v>
       </c>
-      <c r="S13">
+      <c r="S13" s="3">
+        <v>46140.48586303241</v>
+      </c>
+      <c r="T13">
         <v>3</v>
       </c>
-      <c r="T13" s="3">
+      <c r="U13" s="3">
         <v>46131.59102947917</v>
       </c>
     </row>
-    <row r="14" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>63</v>
       </c>
       <c r="B14" t="s">
-        <v>61</v>
+        <v>68</v>
       </c>
       <c r="C14" t="s">
-        <v>62</v>
+        <v>69</v>
       </c>
       <c r="D14" t="s">
-        <v>63</v>
+        <v>70</v>
       </c>
       <c r="F14" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="G14" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="I14">
         <v>12</v>
@@ -1549,51 +1610,54 @@
         <v>46478</v>
       </c>
       <c r="M14" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="N14" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="O14" t="s">
-        <v>23</v>
-      </c>
-      <c r="P14" s="2">
-        <v>170</v>
-      </c>
-      <c r="Q14" s="3">
-        <v>46140.485498043985</v>
+        <v>24</v>
+      </c>
+      <c r="P14" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q14" s="2">
+        <v>2040</v>
       </c>
       <c r="R14" s="3">
         <v>46140.485498043985</v>
       </c>
-      <c r="S14">
+      <c r="S14" s="3">
+        <v>46140.485498043985</v>
+      </c>
+      <c r="T14">
         <v>3</v>
       </c>
-      <c r="T14" s="3">
+      <c r="U14" s="3">
         <v>46131.59056681713</v>
       </c>
     </row>
-    <row r="15" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A15">
         <v>62</v>
       </c>
       <c r="B15" t="s">
-        <v>64</v>
+        <v>71</v>
       </c>
       <c r="C15" t="s">
-        <v>65</v>
+        <v>72</v>
       </c>
       <c r="D15" t="s">
-        <v>66</v>
+        <v>73</v>
       </c>
       <c r="E15" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="F15" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="G15" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="I15">
         <v>12</v>
@@ -1605,48 +1669,51 @@
         <v>46478</v>
       </c>
       <c r="M15" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="N15" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="O15" t="s">
-        <v>23</v>
-      </c>
-      <c r="P15" s="2">
-        <v>220</v>
-      </c>
-      <c r="Q15" s="3">
-        <v>46140.48513407407</v>
+        <v>24</v>
+      </c>
+      <c r="P15" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="Q15" s="2">
+        <v>2640</v>
       </c>
       <c r="R15" s="3">
         <v>46140.48513407407</v>
       </c>
-      <c r="S15">
+      <c r="S15" s="3">
+        <v>46140.48513407407</v>
+      </c>
+      <c r="T15">
         <v>3</v>
       </c>
-      <c r="T15" s="3">
+      <c r="U15" s="3">
         <v>46131.5892174537</v>
       </c>
     </row>
-    <row r="16" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A16">
         <v>61</v>
       </c>
       <c r="B16" t="s">
-        <v>67</v>
+        <v>74</v>
       </c>
       <c r="C16" t="s">
-        <v>68</v>
+        <v>75</v>
       </c>
       <c r="D16" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="F16" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="G16" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="I16">
         <v>12</v>
@@ -1658,51 +1725,54 @@
         <v>46478</v>
       </c>
       <c r="M16" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="N16" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="O16" t="s">
-        <v>23</v>
-      </c>
-      <c r="P16" s="2">
-        <v>170</v>
-      </c>
-      <c r="Q16" s="3">
-        <v>46140.48442474537</v>
+        <v>24</v>
+      </c>
+      <c r="P16" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q16" s="2">
+        <v>2040</v>
       </c>
       <c r="R16" s="3">
         <v>46140.48442474537</v>
       </c>
-      <c r="S16">
+      <c r="S16" s="3">
+        <v>46140.48442474537</v>
+      </c>
+      <c r="T16">
         <v>3</v>
       </c>
-      <c r="T16" s="3">
+      <c r="U16" s="3">
         <v>46131.58870177083</v>
       </c>
     </row>
-    <row r="17" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A17">
         <v>60</v>
       </c>
       <c r="B17" t="s">
-        <v>69</v>
+        <v>76</v>
       </c>
       <c r="C17" t="s">
-        <v>70</v>
+        <v>77</v>
       </c>
       <c r="D17" t="s">
-        <v>71</v>
+        <v>78</v>
       </c>
       <c r="E17" t="s">
-        <v>72</v>
+        <v>79</v>
       </c>
       <c r="F17" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="G17" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="I17">
         <v>12</v>
@@ -1714,96 +1784,102 @@
         <v>46478</v>
       </c>
       <c r="M17" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="N17" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="O17" t="s">
-        <v>23</v>
-      </c>
-      <c r="P17" s="2">
-        <v>220</v>
-      </c>
-      <c r="Q17" s="3">
-        <v>46140.48406033565</v>
+        <v>24</v>
+      </c>
+      <c r="P17" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="Q17" s="2">
+        <v>2640</v>
       </c>
       <c r="R17" s="3">
         <v>46140.48406033565</v>
       </c>
-      <c r="S17">
+      <c r="S17" s="3">
+        <v>46140.48406033565</v>
+      </c>
+      <c r="T17">
         <v>3</v>
       </c>
-      <c r="T17" s="3">
+      <c r="U17" s="3">
         <v>46131.58808645833</v>
       </c>
     </row>
-    <row r="18" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A18">
         <v>59</v>
       </c>
       <c r="B18" t="s">
-        <v>73</v>
+        <v>80</v>
       </c>
       <c r="C18" t="s">
-        <v>74</v>
+        <v>81</v>
       </c>
       <c r="D18" t="s">
-        <v>75</v>
+        <v>82</v>
       </c>
       <c r="E18" t="s">
-        <v>76</v>
+        <v>83</v>
       </c>
       <c r="F18" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="G18" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="J18" s="1"/>
       <c r="K18" s="1"/>
       <c r="M18" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="N18" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="O18" t="s">
-        <v>23</v>
-      </c>
-      <c r="P18" s="2">
+        <v>24</v>
+      </c>
+      <c r="P18" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="Q18" s="2">
         <v>40</v>
       </c>
-      <c r="Q18" s="3"/>
       <c r="R18" s="3"/>
-      <c r="S18">
+      <c r="S18" s="3"/>
+      <c r="T18">
         <v>3</v>
       </c>
-      <c r="T18" s="3">
+      <c r="U18" s="3">
         <v>46131.58666444445</v>
       </c>
     </row>
-    <row r="19" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A19">
         <v>58</v>
       </c>
       <c r="B19" t="s">
-        <v>77</v>
+        <v>84</v>
       </c>
       <c r="C19" t="s">
-        <v>78</v>
+        <v>85</v>
       </c>
       <c r="D19" t="s">
+        <v>86</v>
+      </c>
+      <c r="E19" t="s">
         <v>79</v>
       </c>
-      <c r="E19" t="s">
-        <v>72</v>
-      </c>
       <c r="F19" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="G19" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="I19">
         <v>12</v>
@@ -1815,84 +1891,90 @@
         <v>46479</v>
       </c>
       <c r="M19" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="N19" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="O19" t="s">
-        <v>23</v>
-      </c>
-      <c r="P19" s="2">
-        <v>170</v>
-      </c>
-      <c r="Q19" s="3">
-        <v>46140.48369461806</v>
+        <v>24</v>
+      </c>
+      <c r="P19" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q19" s="2">
+        <v>2040</v>
       </c>
       <c r="R19" s="3">
         <v>46140.48369461806</v>
       </c>
-      <c r="S19">
+      <c r="S19" s="3">
+        <v>46140.48369461806</v>
+      </c>
+      <c r="T19">
         <v>3</v>
       </c>
-      <c r="T19" s="3">
+      <c r="U19" s="3">
         <v>46131.58577715278</v>
       </c>
     </row>
-    <row r="20" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A20">
         <v>57</v>
       </c>
       <c r="B20" t="s">
-        <v>80</v>
+        <v>87</v>
       </c>
       <c r="C20" t="s">
-        <v>81</v>
+        <v>88</v>
       </c>
       <c r="D20" t="s">
-        <v>82</v>
+        <v>89</v>
       </c>
       <c r="E20" t="s">
-        <v>72</v>
+        <v>79</v>
       </c>
       <c r="F20" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="J20" s="1"/>
       <c r="K20" s="1"/>
-      <c r="P20" s="2">
+      <c r="P20" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="Q20" s="2">
         <v>0</v>
       </c>
-      <c r="Q20" s="3"/>
       <c r="R20" s="3"/>
-      <c r="S20">
+      <c r="S20" s="3"/>
+      <c r="T20">
         <v>3</v>
       </c>
-      <c r="T20" s="3">
+      <c r="U20" s="3">
         <v>46131.585335868054</v>
       </c>
     </row>
-    <row r="21" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A21">
         <v>55</v>
       </c>
       <c r="B21" t="s">
-        <v>83</v>
+        <v>90</v>
       </c>
       <c r="C21" t="s">
-        <v>84</v>
+        <v>91</v>
       </c>
       <c r="D21" t="s">
-        <v>85</v>
+        <v>92</v>
       </c>
       <c r="E21" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="F21" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="G21" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="I21">
         <v>12</v>
@@ -1904,48 +1986,51 @@
         <v>46479</v>
       </c>
       <c r="M21" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="N21" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="O21" t="s">
-        <v>23</v>
-      </c>
-      <c r="P21" s="2">
-        <v>220</v>
-      </c>
-      <c r="Q21" s="3">
-        <v>46140.48327597222</v>
+        <v>24</v>
+      </c>
+      <c r="P21" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="Q21" s="2">
+        <v>2640</v>
       </c>
       <c r="R21" s="3">
         <v>46140.48327597222</v>
       </c>
-      <c r="S21">
+      <c r="S21" s="3">
+        <v>46140.48327597222</v>
+      </c>
+      <c r="T21">
         <v>3</v>
       </c>
-      <c r="T21" s="3">
+      <c r="U21" s="3">
         <v>46131.58447693287</v>
       </c>
     </row>
-    <row r="22" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A22">
         <v>54</v>
       </c>
       <c r="B22" t="s">
-        <v>86</v>
+        <v>93</v>
       </c>
       <c r="C22" t="s">
-        <v>87</v>
+        <v>94</v>
       </c>
       <c r="D22" t="s">
-        <v>88</v>
+        <v>95</v>
       </c>
       <c r="F22" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="G22" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="I22">
         <v>12</v>
@@ -1957,48 +2042,51 @@
         <v>46479</v>
       </c>
       <c r="M22" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="N22" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="O22" t="s">
-        <v>23</v>
-      </c>
-      <c r="P22" s="2">
-        <v>210</v>
-      </c>
-      <c r="Q22" s="3">
-        <v>46140.48291085648</v>
+        <v>24</v>
+      </c>
+      <c r="P22" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="Q22" s="2">
+        <v>2630</v>
       </c>
       <c r="R22" s="3">
         <v>46140.48291085648</v>
       </c>
-      <c r="S22">
+      <c r="S22" s="3">
+        <v>46140.48291085648</v>
+      </c>
+      <c r="T22">
         <v>3</v>
       </c>
-      <c r="T22" s="3">
+      <c r="U22" s="3">
         <v>46131.58377670139</v>
       </c>
     </row>
-    <row r="23" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A23">
         <v>53</v>
       </c>
       <c r="B23" t="s">
-        <v>89</v>
+        <v>96</v>
       </c>
       <c r="C23" t="s">
-        <v>90</v>
+        <v>97</v>
       </c>
       <c r="D23" t="s">
-        <v>91</v>
+        <v>98</v>
       </c>
       <c r="F23" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="G23" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="I23">
         <v>12</v>
@@ -2010,48 +2098,51 @@
         <v>46479</v>
       </c>
       <c r="M23" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="N23" t="s">
-        <v>92</v>
+        <v>99</v>
       </c>
       <c r="O23" t="s">
-        <v>93</v>
-      </c>
-      <c r="P23" s="2">
-        <v>210</v>
-      </c>
-      <c r="Q23" s="3">
-        <v>46140.48255181713</v>
+        <v>100</v>
+      </c>
+      <c r="P23" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="Q23" s="2">
+        <v>2630</v>
       </c>
       <c r="R23" s="3">
         <v>46140.48255181713</v>
       </c>
-      <c r="S23">
+      <c r="S23" s="3">
+        <v>46140.48255181713</v>
+      </c>
+      <c r="T23">
         <v>3</v>
       </c>
-      <c r="T23" s="3">
+      <c r="U23" s="3">
         <v>46131.58282542824</v>
       </c>
     </row>
-    <row r="24" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A24">
         <v>52</v>
       </c>
       <c r="B24" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="C24" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="D24" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="F24" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="G24" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="I24">
         <v>12</v>
@@ -2063,48 +2154,51 @@
         <v>46478</v>
       </c>
       <c r="M24" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="N24" t="s">
-        <v>94</v>
+        <v>101</v>
       </c>
       <c r="O24" t="s">
-        <v>95</v>
-      </c>
-      <c r="P24" s="2">
-        <v>210</v>
-      </c>
-      <c r="Q24" s="3">
-        <v>46140.481821863425</v>
+        <v>102</v>
+      </c>
+      <c r="P24" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="Q24" s="2">
+        <v>2630</v>
       </c>
       <c r="R24" s="3">
         <v>46140.481821863425</v>
       </c>
-      <c r="S24">
+      <c r="S24" s="3">
+        <v>46140.481821863425</v>
+      </c>
+      <c r="T24">
         <v>3</v>
       </c>
-      <c r="T24" s="3">
+      <c r="U24" s="3">
         <v>46131.58113885416</v>
       </c>
     </row>
-    <row r="25" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A25">
         <v>51</v>
       </c>
       <c r="B25" t="s">
-        <v>96</v>
+        <v>103</v>
       </c>
       <c r="C25" t="s">
-        <v>97</v>
+        <v>104</v>
       </c>
       <c r="D25" t="s">
-        <v>98</v>
+        <v>105</v>
       </c>
       <c r="F25" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="G25" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="I25">
         <v>12</v>
@@ -2116,48 +2210,51 @@
         <v>46478</v>
       </c>
       <c r="M25" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="N25" t="s">
-        <v>99</v>
+        <v>106</v>
       </c>
       <c r="O25" t="s">
-        <v>100</v>
-      </c>
-      <c r="P25" s="2">
-        <v>170</v>
-      </c>
-      <c r="Q25" s="3">
-        <v>46140.48145364583</v>
+        <v>107</v>
+      </c>
+      <c r="P25" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q25" s="2">
+        <v>2040</v>
       </c>
       <c r="R25" s="3">
         <v>46140.48145364583</v>
       </c>
-      <c r="S25">
+      <c r="S25" s="3">
+        <v>46140.48145364583</v>
+      </c>
+      <c r="T25">
         <v>3</v>
       </c>
-      <c r="T25" s="3">
+      <c r="U25" s="3">
         <v>46131.57980773148</v>
       </c>
     </row>
-    <row r="26" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A26">
         <v>50</v>
       </c>
       <c r="B26" t="s">
-        <v>101</v>
+        <v>108</v>
       </c>
       <c r="C26" t="s">
-        <v>102</v>
+        <v>109</v>
       </c>
       <c r="D26" t="s">
-        <v>103</v>
+        <v>110</v>
       </c>
       <c r="F26" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="G26" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="I26">
         <v>12</v>
@@ -2169,51 +2266,54 @@
         <v>46478</v>
       </c>
       <c r="M26" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="N26" t="s">
-        <v>104</v>
+        <v>111</v>
       </c>
       <c r="O26" t="s">
-        <v>105</v>
-      </c>
-      <c r="P26" s="2">
-        <v>220</v>
-      </c>
-      <c r="Q26" s="3">
-        <v>46140.48109398148</v>
+        <v>112</v>
+      </c>
+      <c r="P26" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="Q26" s="2">
+        <v>2640</v>
       </c>
       <c r="R26" s="3">
         <v>46140.48109398148</v>
       </c>
-      <c r="S26">
+      <c r="S26" s="3">
+        <v>46140.48109398148</v>
+      </c>
+      <c r="T26">
         <v>3</v>
       </c>
-      <c r="T26" s="3">
+      <c r="U26" s="3">
         <v>46131.57757702546</v>
       </c>
     </row>
-    <row r="27" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A27">
         <v>49</v>
       </c>
       <c r="B27" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C27" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="D27" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="E27" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="F27" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="G27" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="H27">
         <v>12</v>
@@ -2227,40 +2327,43 @@
       <c r="K27" s="1">
         <v>46478</v>
       </c>
-      <c r="P27" s="2">
-        <v>1180</v>
-      </c>
-      <c r="Q27" s="3">
-        <v>46140.48058773148</v>
+      <c r="P27" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q27" s="2">
+        <v>3050</v>
       </c>
       <c r="R27" s="3">
         <v>46140.48058773148</v>
       </c>
-      <c r="S27">
+      <c r="S27" s="3">
+        <v>46140.48058773148</v>
+      </c>
+      <c r="T27">
         <v>3</v>
       </c>
-      <c r="T27" s="3">
+      <c r="U27" s="3">
         <v>46122.751813842595</v>
       </c>
     </row>
-    <row r="28" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A28">
         <v>47</v>
       </c>
       <c r="B28" t="s">
-        <v>106</v>
+        <v>113</v>
       </c>
       <c r="C28" t="s">
-        <v>107</v>
+        <v>114</v>
       </c>
       <c r="D28" t="s">
-        <v>108</v>
+        <v>115</v>
       </c>
       <c r="F28" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="G28" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="I28">
         <v>12</v>
@@ -2272,126 +2375,135 @@
         <v>46478</v>
       </c>
       <c r="M28" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="N28" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="O28" t="s">
-        <v>23</v>
-      </c>
-      <c r="P28" s="2">
-        <v>220</v>
-      </c>
-      <c r="Q28" s="3">
-        <v>46140.47577868056</v>
+        <v>24</v>
+      </c>
+      <c r="P28" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="Q28" s="2">
+        <v>2640</v>
       </c>
       <c r="R28" s="3">
         <v>46140.47577868056</v>
       </c>
-      <c r="S28">
+      <c r="S28" s="3">
+        <v>46140.47577868056</v>
+      </c>
+      <c r="T28">
         <v>3</v>
       </c>
-      <c r="T28" s="3">
+      <c r="U28" s="3">
         <v>46116.09188155092</v>
       </c>
     </row>
-    <row r="29" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A29">
         <v>42</v>
       </c>
       <c r="B29" t="s">
-        <v>109</v>
+        <v>116</v>
       </c>
       <c r="C29" t="s">
-        <v>110</v>
+        <v>117</v>
       </c>
       <c r="D29" t="s">
-        <v>111</v>
+        <v>118</v>
       </c>
       <c r="E29" t="s">
-        <v>112</v>
+        <v>119</v>
       </c>
       <c r="F29" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="G29" t="s">
-        <v>113</v>
+        <v>120</v>
       </c>
       <c r="J29" s="1">
         <v>46029</v>
       </c>
       <c r="K29" s="1"/>
       <c r="M29" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="N29" t="s">
-        <v>114</v>
+        <v>121</v>
       </c>
       <c r="O29" t="s">
-        <v>115</v>
-      </c>
-      <c r="P29" s="2">
+        <v>122</v>
+      </c>
+      <c r="P29" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="Q29" s="2">
         <v>0</v>
       </c>
-      <c r="Q29" s="3"/>
       <c r="R29" s="3"/>
-      <c r="S29">
+      <c r="S29" s="3"/>
+      <c r="T29">
         <v>3</v>
       </c>
-      <c r="T29" s="3">
+      <c r="U29" s="3">
         <v>46109.901882743055</v>
       </c>
     </row>
-    <row r="30" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A30">
         <v>41</v>
       </c>
       <c r="B30" t="s">
-        <v>116</v>
+        <v>123</v>
       </c>
       <c r="C30" t="s">
-        <v>117</v>
+        <v>124</v>
       </c>
       <c r="D30" t="s">
-        <v>118</v>
+        <v>125</v>
       </c>
       <c r="E30" t="s">
-        <v>119</v>
+        <v>126</v>
       </c>
       <c r="F30" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="G30" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="J30" s="1">
         <v>46107</v>
       </c>
       <c r="K30" s="1"/>
       <c r="M30" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="N30" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="O30" t="s">
-        <v>121</v>
-      </c>
-      <c r="P30" s="2">
+        <v>128</v>
+      </c>
+      <c r="P30" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="Q30" s="2">
         <v>70</v>
       </c>
-      <c r="Q30" s="3"/>
       <c r="R30" s="3"/>
-      <c r="S30">
+      <c r="S30" s="3"/>
+      <c r="T30">
         <v>3</v>
       </c>
-      <c r="T30" s="3">
+      <c r="U30" s="3">
         <v>46108.11050890046</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:T1"/>
+  <autoFilter ref="A1:U1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
@@ -2399,7 +2511,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:O13"/>
+  <dimension ref="A1:P13"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="8" customWidth="1"/>
@@ -2412,72 +2524,76 @@
     <col min="9" max="10" width="12" customWidth="1"/>
     <col min="11" max="12" width="14" style="2" customWidth="1"/>
     <col min="13" max="13" width="12" style="2" customWidth="1"/>
-    <col min="14" max="14" width="16" style="2" customWidth="1"/>
-    <col min="15" max="15" width="30" customWidth="1"/>
+    <col min="14" max="14" width="18" style="2" customWidth="1"/>
+    <col min="15" max="15" width="16" style="2" customWidth="1"/>
+    <col min="16" max="16" width="30" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="22" customHeight="1" spans="1:15" s="4" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" ht="22" customHeight="1" spans="1:16" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
-        <v>122</v>
+        <v>129</v>
       </c>
       <c r="B1" s="4" t="s">
         <v>1</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>123</v>
+        <v>130</v>
       </c>
       <c r="D1" s="4" t="s">
-        <v>124</v>
+        <v>131</v>
       </c>
       <c r="E1" s="4" t="s">
-        <v>125</v>
+        <v>132</v>
       </c>
       <c r="F1" s="4" t="s">
-        <v>126</v>
+        <v>133</v>
       </c>
       <c r="G1" s="4" t="s">
-        <v>127</v>
+        <v>134</v>
       </c>
       <c r="H1" s="4" t="s">
-        <v>128</v>
+        <v>135</v>
       </c>
       <c r="I1" s="4" t="s">
-        <v>129</v>
+        <v>136</v>
       </c>
       <c r="J1" s="4" t="s">
-        <v>130</v>
+        <v>137</v>
       </c>
       <c r="K1" s="6" t="s">
-        <v>131</v>
+        <v>138</v>
       </c>
       <c r="L1" s="6" t="s">
-        <v>132</v>
+        <v>139</v>
       </c>
       <c r="M1" s="6" t="s">
-        <v>133</v>
+        <v>140</v>
       </c>
       <c r="N1" s="6" t="s">
-        <v>134</v>
-      </c>
-      <c r="O1" s="4" t="s">
-        <v>135</v>
-      </c>
-    </row>
-    <row r="2" spans="1:15" x14ac:dyDescent="0.25">
+        <v>15</v>
+      </c>
+      <c r="O1" s="6" t="s">
+        <v>141</v>
+      </c>
+      <c r="P1" s="4" t="s">
+        <v>142</v>
+      </c>
+    </row>
+    <row r="2" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>41</v>
       </c>
       <c r="B2" t="s">
-        <v>116</v>
+        <v>123</v>
       </c>
       <c r="C2" t="s">
-        <v>136</v>
+        <v>143</v>
       </c>
       <c r="D2" t="s">
-        <v>137</v>
+        <v>144</v>
       </c>
       <c r="E2" t="s">
-        <v>138</v>
+        <v>145</v>
       </c>
       <c r="H2">
         <v>1</v>
@@ -2489,25 +2605,26 @@
       <c r="M2" s="2">
         <v>10</v>
       </c>
-      <c r="N2" s="2">
+      <c r="N2" s="2"/>
+      <c r="O2" s="2">
         <v>70</v>
       </c>
     </row>
-    <row r="3" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>49</v>
       </c>
       <c r="B3" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C3" t="s">
-        <v>139</v>
+        <v>146</v>
       </c>
       <c r="D3" t="s">
-        <v>137</v>
+        <v>144</v>
       </c>
       <c r="E3" t="s">
-        <v>138</v>
+        <v>145</v>
       </c>
       <c r="H3">
         <v>1</v>
@@ -2522,25 +2639,26 @@
       <c r="M3" s="2">
         <v>80</v>
       </c>
-      <c r="N3" s="2">
+      <c r="N3" s="2"/>
+      <c r="O3" s="2">
         <v>720</v>
       </c>
     </row>
-    <row r="4" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>49</v>
       </c>
       <c r="B4" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C4" t="s">
-        <v>140</v>
+        <v>147</v>
       </c>
       <c r="D4" t="s">
-        <v>141</v>
+        <v>148</v>
       </c>
       <c r="E4" t="s">
-        <v>138</v>
+        <v>145</v>
       </c>
       <c r="H4">
         <v>1</v>
@@ -2555,25 +2673,26 @@
       <c r="M4" s="2">
         <v>10</v>
       </c>
-      <c r="N4" s="2">
+      <c r="N4" s="2"/>
+      <c r="O4" s="2">
         <v>290</v>
       </c>
     </row>
-    <row r="5" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>59</v>
       </c>
       <c r="B5" t="s">
-        <v>73</v>
+        <v>80</v>
       </c>
       <c r="C5" t="s">
-        <v>142</v>
+        <v>149</v>
       </c>
       <c r="D5" t="s">
-        <v>143</v>
+        <v>150</v>
       </c>
       <c r="E5" t="s">
-        <v>144</v>
+        <v>151</v>
       </c>
       <c r="H5">
         <v>1</v>
@@ -2585,25 +2704,26 @@
       <c r="M5" s="2">
         <v>10</v>
       </c>
-      <c r="N5" s="2">
+      <c r="N5" s="2"/>
+      <c r="O5" s="2">
         <v>40</v>
       </c>
     </row>
-    <row r="6" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>68</v>
       </c>
       <c r="B6" t="s">
-        <v>46</v>
+        <v>50</v>
       </c>
       <c r="C6" t="s">
-        <v>142</v>
+        <v>149</v>
       </c>
       <c r="D6" t="s">
-        <v>143</v>
+        <v>150</v>
       </c>
       <c r="E6" t="s">
-        <v>144</v>
+        <v>151</v>
       </c>
       <c r="H6">
         <v>1</v>
@@ -2615,25 +2735,26 @@
       <c r="M6" s="2">
         <v>10</v>
       </c>
-      <c r="N6" s="2">
+      <c r="N6" s="2"/>
+      <c r="O6" s="2">
         <v>40</v>
       </c>
     </row>
-    <row r="7" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>70</v>
       </c>
       <c r="B7" t="s">
-        <v>41</v>
+        <v>45</v>
       </c>
       <c r="C7" t="s">
-        <v>139</v>
+        <v>146</v>
       </c>
       <c r="D7" t="s">
-        <v>137</v>
+        <v>144</v>
       </c>
       <c r="E7" t="s">
-        <v>138</v>
+        <v>145</v>
       </c>
       <c r="H7">
         <v>2</v>
@@ -2648,25 +2769,26 @@
       <c r="M7" s="2">
         <v>100</v>
       </c>
-      <c r="N7" s="2">
+      <c r="N7" s="2"/>
+      <c r="O7" s="2">
         <v>700</v>
       </c>
     </row>
-    <row r="8" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>72</v>
       </c>
       <c r="B8" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="C8" t="s">
-        <v>136</v>
+        <v>143</v>
       </c>
       <c r="D8" t="s">
-        <v>137</v>
+        <v>144</v>
       </c>
       <c r="E8" t="s">
-        <v>138</v>
+        <v>145</v>
       </c>
       <c r="H8">
         <v>2</v>
@@ -2678,25 +2800,26 @@
       <c r="M8" s="2">
         <v>0</v>
       </c>
-      <c r="N8" s="2">
+      <c r="N8" s="2"/>
+      <c r="O8" s="2">
         <v>80</v>
       </c>
     </row>
-    <row r="9" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>73</v>
       </c>
       <c r="B9" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="C9" t="s">
-        <v>136</v>
+        <v>143</v>
       </c>
       <c r="D9" t="s">
-        <v>137</v>
+        <v>144</v>
       </c>
       <c r="E9" t="s">
-        <v>138</v>
+        <v>145</v>
       </c>
       <c r="H9">
         <v>1</v>
@@ -2708,25 +2831,26 @@
       <c r="M9" s="2">
         <v>0</v>
       </c>
-      <c r="N9" s="2">
+      <c r="N9" s="2"/>
+      <c r="O9" s="2">
         <v>80</v>
       </c>
     </row>
-    <row r="10" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>74</v>
       </c>
       <c r="B10" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C10" t="s">
+        <v>152</v>
+      </c>
+      <c r="D10" t="s">
+        <v>148</v>
+      </c>
+      <c r="E10" t="s">
         <v>145</v>
-      </c>
-      <c r="D10" t="s">
-        <v>141</v>
-      </c>
-      <c r="E10" t="s">
-        <v>138</v>
       </c>
       <c r="H10">
         <v>1</v>
@@ -2738,25 +2862,26 @@
       <c r="M10" s="2">
         <v>0</v>
       </c>
-      <c r="N10" s="2">
+      <c r="N10" s="2"/>
+      <c r="O10" s="2">
         <v>120</v>
       </c>
     </row>
-    <row r="11" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>75</v>
       </c>
       <c r="B11" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="C11" t="s">
+        <v>152</v>
+      </c>
+      <c r="D11" t="s">
+        <v>148</v>
+      </c>
+      <c r="E11" t="s">
         <v>145</v>
-      </c>
-      <c r="D11" t="s">
-        <v>141</v>
-      </c>
-      <c r="E11" t="s">
-        <v>138</v>
       </c>
       <c r="H11">
         <v>2</v>
@@ -2768,25 +2893,26 @@
       <c r="M11" s="2">
         <v>0</v>
       </c>
-      <c r="N11" s="2">
+      <c r="N11" s="2"/>
+      <c r="O11" s="2">
         <v>120</v>
       </c>
     </row>
-    <row r="12" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>76</v>
       </c>
       <c r="B12" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C12" t="s">
-        <v>146</v>
+        <v>153</v>
       </c>
       <c r="D12" t="s">
-        <v>141</v>
+        <v>148</v>
       </c>
       <c r="E12" t="s">
-        <v>138</v>
+        <v>145</v>
       </c>
       <c r="H12">
         <v>1</v>
@@ -2798,25 +2924,26 @@
       <c r="M12" s="2">
         <v>0</v>
       </c>
-      <c r="N12" s="2">
+      <c r="N12" s="2"/>
+      <c r="O12" s="2">
         <v>120</v>
       </c>
     </row>
-    <row r="13" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>76</v>
       </c>
       <c r="B13" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C13" t="s">
-        <v>147</v>
+        <v>154</v>
       </c>
       <c r="D13" t="s">
-        <v>141</v>
+        <v>148</v>
       </c>
       <c r="E13" t="s">
-        <v>138</v>
+        <v>145</v>
       </c>
       <c r="H13">
         <v>2</v>
@@ -2828,12 +2955,13 @@
       <c r="M13" s="2">
         <v>0</v>
       </c>
-      <c r="N13" s="2">
+      <c r="N13" s="2"/>
+      <c r="O13" s="2">
         <v>80</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:O1"/>
+  <autoFilter ref="A1:P1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
@@ -2853,7 +2981,7 @@
   <sheetData>
     <row r="1" ht="22" customHeight="1" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
-        <v>122</v>
+        <v>129</v>
       </c>
       <c r="B1" s="4" t="s">
         <v>1</v>
@@ -2862,10 +2990,10 @@
         <v>5</v>
       </c>
       <c r="D1" s="4" t="s">
-        <v>148</v>
+        <v>155</v>
       </c>
       <c r="E1" s="6" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
@@ -2873,16 +3001,16 @@
         <v>76</v>
       </c>
       <c r="B2" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C2" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="D2" t="s">
-        <v>149</v>
+        <v>156</v>
       </c>
       <c r="E2" s="2">
-        <v>370</v>
+        <v>2240</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
@@ -2890,16 +3018,16 @@
         <v>75</v>
       </c>
       <c r="B3" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="C3" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="D3" t="s">
-        <v>145</v>
+        <v>152</v>
       </c>
       <c r="E3" s="2">
-        <v>290</v>
+        <v>2160</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
@@ -2907,16 +3035,16 @@
         <v>74</v>
       </c>
       <c r="B4" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C4" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="D4" t="s">
-        <v>145</v>
+        <v>152</v>
       </c>
       <c r="E4" s="2">
-        <v>290</v>
+        <v>2160</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
@@ -2924,13 +3052,13 @@
         <v>73</v>
       </c>
       <c r="B5" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="C5" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="D5" t="s">
-        <v>136</v>
+        <v>143</v>
       </c>
       <c r="E5" s="2">
         <v>80</v>
@@ -2941,13 +3069,13 @@
         <v>72</v>
       </c>
       <c r="B6" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="C6" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="D6" t="s">
-        <v>136</v>
+        <v>143</v>
       </c>
       <c r="E6" s="2">
         <v>80</v>
@@ -2958,16 +3086,16 @@
         <v>71</v>
       </c>
       <c r="B7" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="C7" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="D7" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E7" s="2">
-        <v>160</v>
+        <v>2030</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
@@ -2975,13 +3103,13 @@
         <v>70</v>
       </c>
       <c r="B8" t="s">
-        <v>41</v>
+        <v>45</v>
       </c>
       <c r="C8" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="D8" t="s">
-        <v>139</v>
+        <v>146</v>
       </c>
       <c r="E8" s="2">
         <v>700</v>
@@ -2992,13 +3120,13 @@
         <v>68</v>
       </c>
       <c r="B9" t="s">
-        <v>46</v>
+        <v>50</v>
       </c>
       <c r="C9" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="D9" t="s">
-        <v>142</v>
+        <v>149</v>
       </c>
       <c r="E9" s="2">
         <v>40</v>
@@ -3009,16 +3137,16 @@
         <v>67</v>
       </c>
       <c r="B10" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="C10" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="D10" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E10" s="2">
-        <v>210</v>
+        <v>2630</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
@@ -3026,16 +3154,16 @@
         <v>66</v>
       </c>
       <c r="B11" t="s">
-        <v>51</v>
+        <v>56</v>
       </c>
       <c r="C11" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="D11" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E11" s="2">
-        <v>160</v>
+        <v>2030</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
@@ -3043,16 +3171,16 @@
         <v>65</v>
       </c>
       <c r="B12" t="s">
-        <v>54</v>
+        <v>59</v>
       </c>
       <c r="C12" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="D12" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E12" s="2">
-        <v>200</v>
+        <v>2620</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">
@@ -3060,16 +3188,16 @@
         <v>64</v>
       </c>
       <c r="B13" t="s">
-        <v>59</v>
+        <v>65</v>
       </c>
       <c r="C13" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="D13" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E13" s="2">
-        <v>220</v>
+        <v>2640</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.25">
@@ -3077,16 +3205,16 @@
         <v>63</v>
       </c>
       <c r="B14" t="s">
-        <v>61</v>
+        <v>68</v>
       </c>
       <c r="C14" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="D14" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E14" s="2">
-        <v>170</v>
+        <v>2040</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.25">
@@ -3094,16 +3222,16 @@
         <v>62</v>
       </c>
       <c r="B15" t="s">
-        <v>64</v>
+        <v>71</v>
       </c>
       <c r="C15" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="D15" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E15" s="2">
-        <v>220</v>
+        <v>2640</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.25">
@@ -3111,16 +3239,16 @@
         <v>61</v>
       </c>
       <c r="B16" t="s">
-        <v>67</v>
+        <v>74</v>
       </c>
       <c r="C16" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="D16" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E16" s="2">
-        <v>170</v>
+        <v>2040</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.25">
@@ -3128,16 +3256,16 @@
         <v>60</v>
       </c>
       <c r="B17" t="s">
-        <v>69</v>
+        <v>76</v>
       </c>
       <c r="C17" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="D17" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E17" s="2">
-        <v>220</v>
+        <v>2640</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.25">
@@ -3145,13 +3273,13 @@
         <v>59</v>
       </c>
       <c r="B18" t="s">
-        <v>73</v>
+        <v>80</v>
       </c>
       <c r="C18" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="D18" t="s">
-        <v>142</v>
+        <v>149</v>
       </c>
       <c r="E18" s="2">
         <v>40</v>
@@ -3162,16 +3290,16 @@
         <v>58</v>
       </c>
       <c r="B19" t="s">
-        <v>77</v>
+        <v>84</v>
       </c>
       <c r="C19" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="D19" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E19" s="2">
-        <v>170</v>
+        <v>2040</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.25">
@@ -3179,13 +3307,13 @@
         <v>57</v>
       </c>
       <c r="B20" t="s">
-        <v>80</v>
+        <v>87</v>
       </c>
       <c r="C20" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="D20" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E20" s="2">
         <v>0</v>
@@ -3196,16 +3324,16 @@
         <v>55</v>
       </c>
       <c r="B21" t="s">
-        <v>83</v>
+        <v>90</v>
       </c>
       <c r="C21" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="D21" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E21" s="2">
-        <v>220</v>
+        <v>2640</v>
       </c>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.25">
@@ -3213,16 +3341,16 @@
         <v>54</v>
       </c>
       <c r="B22" t="s">
-        <v>86</v>
+        <v>93</v>
       </c>
       <c r="C22" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="D22" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E22" s="2">
-        <v>210</v>
+        <v>2630</v>
       </c>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.25">
@@ -3230,16 +3358,16 @@
         <v>53</v>
       </c>
       <c r="B23" t="s">
-        <v>89</v>
+        <v>96</v>
       </c>
       <c r="C23" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="D23" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E23" s="2">
-        <v>210</v>
+        <v>2630</v>
       </c>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.25">
@@ -3247,16 +3375,16 @@
         <v>52</v>
       </c>
       <c r="B24" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="C24" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="D24" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E24" s="2">
-        <v>210</v>
+        <v>2630</v>
       </c>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.25">
@@ -3264,16 +3392,16 @@
         <v>51</v>
       </c>
       <c r="B25" t="s">
-        <v>96</v>
+        <v>103</v>
       </c>
       <c r="C25" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="D25" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E25" s="2">
-        <v>170</v>
+        <v>2040</v>
       </c>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.25">
@@ -3281,16 +3409,16 @@
         <v>50</v>
       </c>
       <c r="B26" t="s">
-        <v>101</v>
+        <v>108</v>
       </c>
       <c r="C26" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="D26" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E26" s="2">
-        <v>220</v>
+        <v>2640</v>
       </c>
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.25">
@@ -3298,16 +3426,16 @@
         <v>49</v>
       </c>
       <c r="B27" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C27" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="D27" t="s">
-        <v>150</v>
+        <v>157</v>
       </c>
       <c r="E27" s="2">
-        <v>1180</v>
+        <v>3050</v>
       </c>
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.25">
@@ -3315,16 +3443,16 @@
         <v>47</v>
       </c>
       <c r="B28" t="s">
-        <v>106</v>
+        <v>113</v>
       </c>
       <c r="C28" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="D28" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E28" s="2">
-        <v>220</v>
+        <v>2640</v>
       </c>
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.25">
@@ -3332,13 +3460,13 @@
         <v>42</v>
       </c>
       <c r="B29" t="s">
-        <v>109</v>
+        <v>116</v>
       </c>
       <c r="C29" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="D29" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E29" s="2">
         <v>0</v>
@@ -3349,13 +3477,13 @@
         <v>41</v>
       </c>
       <c r="B30" t="s">
-        <v>116</v>
+        <v>123</v>
       </c>
       <c r="C30" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="D30" t="s">
-        <v>136</v>
+        <v>143</v>
       </c>
       <c r="E30" s="2">
         <v>70</v>

</xml_diff>